<commit_message>
Set transactions status updated
</commit_message>
<xml_diff>
--- a/Data/Config.xlsx
+++ b/Data/Config.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\aci-con2\Documents\UiPath\AMP_R3_RT_MAP\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6A5EFC49-8EAE-4EF4-98C0-C4BECA381457}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{85914B22-EFFD-4B6E-A335-D2CC39D648B6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15195" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -17,19 +17,8 @@
     <sheet name="Constants" sheetId="2" r:id="rId2"/>
     <sheet name="Assets" sheetId="3" r:id="rId3"/>
   </sheets>
-  <calcPr calcId="191029"/>
+  <calcPr calcId="181029"/>
   <extLst>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:Single"/>
-        <xcalcf:feature name="microsoft.com:FV"/>
-        <xcalcf:feature name="microsoft.com:CNMTM"/>
-        <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
-      </xcalcf:calcFeatures>
-    </ext>
     <ext uri="GoogleSheetsCustomDataVersion2">
       <go:sheetsCustomData xmlns:go="http://customooxmlschemas.google.com/" r:id="rId7" roundtripDataChecksum="54QOzkJ5yUFRx/cu0Hfc+S94/d7KJAOULguWs82GEDY="/>
     </ext>

</xml_diff>